<commit_message>
update data2026.xlsx with modified content
</commit_message>
<xml_diff>
--- a/data2026.xlsx
+++ b/data2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\melan\DESU_DATA_2026\ProjetNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CA52BF-E62D-453E-BF93-84A66E69BA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44273B67-B6B7-41EB-8950-54CC0F6F0D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{A5577CF9-A2EC-4381-9165-1BFB57234FC3}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5872" uniqueCount="661">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5864" uniqueCount="661">
   <si>
     <t>Patient</t>
   </si>
@@ -8895,7 +8895,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9E9E3CB-BB82-4E38-9625-63F9049E9733}">
-  <dimension ref="A1:S86"/>
+  <dimension ref="A1:R86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.453125" style="51" bestFit="1" customWidth="1"/>
@@ -8916,7 +8916,7 @@
     <col min="19" max="19" width="31.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8972,7 +8972,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -9027,11 +9027,8 @@
       <c r="R2" s="126" t="s">
         <v>554</v>
       </c>
-      <c r="S2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="51" t="s">
         <v>8</v>
       </c>
@@ -9086,11 +9083,8 @@
       <c r="R3" s="126" t="s">
         <v>552</v>
       </c>
-      <c r="S3" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>69</v>
       </c>
@@ -9145,11 +9139,8 @@
       <c r="R4" s="126" t="s">
         <v>555</v>
       </c>
-      <c r="S4" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="51" t="s">
         <v>29</v>
       </c>
@@ -9204,11 +9195,8 @@
       <c r="R5" s="126" t="s">
         <v>556</v>
       </c>
-      <c r="S5" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="51" t="s">
         <v>30</v>
       </c>
@@ -9263,11 +9251,8 @@
       <c r="R6" s="126" t="s">
         <v>556</v>
       </c>
-      <c r="S6" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="51" t="s">
         <v>12</v>
       </c>
@@ -9322,11 +9307,8 @@
       <c r="R7" s="126" t="s">
         <v>559</v>
       </c>
-      <c r="S7" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="51" t="s">
         <v>14</v>
       </c>
@@ -9381,11 +9363,8 @@
       <c r="R8" s="126" t="s">
         <v>560</v>
       </c>
-      <c r="S8" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="51" t="s">
         <v>31</v>
       </c>
@@ -9440,11 +9419,8 @@
       <c r="R9" s="127" t="s">
         <v>552</v>
       </c>
-      <c r="S9" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="51" t="s">
         <v>33</v>
       </c>
@@ -9500,7 +9476,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="51" t="s">
         <v>35</v>
       </c>
@@ -9556,7 +9532,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="51" t="s">
         <v>37</v>
       </c>
@@ -9612,7 +9588,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="51" t="s">
         <v>38</v>
       </c>
@@ -9668,7 +9644,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="51" t="s">
         <v>39</v>
       </c>
@@ -9724,7 +9700,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="51" t="s">
         <v>40</v>
       </c>
@@ -9780,7 +9756,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="51" t="s">
         <v>25</v>
       </c>

</xml_diff>

<commit_message>
update data2026.xlsx with changes
</commit_message>
<xml_diff>
--- a/data2026.xlsx
+++ b/data2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\melan\DESU_DATA_2026\ProjetNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44273B67-B6B7-41EB-8950-54CC0F6F0D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D96EF0-DBA9-407E-A71D-4F8CBAAF8E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{A5577CF9-A2EC-4381-9165-1BFB57234FC3}"/>
   </bookViews>
@@ -9078,10 +9078,10 @@
         <v>103</v>
       </c>
       <c r="Q3" s="126" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R3" s="126" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
@@ -9414,10 +9414,10 @@
         <v>118</v>
       </c>
       <c r="Q9" s="127" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R9" s="127" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
@@ -9582,10 +9582,10 @@
         <v>72</v>
       </c>
       <c r="Q12" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R12" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
@@ -9638,10 +9638,10 @@
         <v>72</v>
       </c>
       <c r="Q13" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R13" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -9694,10 +9694,10 @@
         <v>97</v>
       </c>
       <c r="Q14" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R14" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
@@ -9750,10 +9750,10 @@
         <v>97</v>
       </c>
       <c r="Q15" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R15" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -9806,10 +9806,10 @@
         <v>112</v>
       </c>
       <c r="Q16" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R16" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
@@ -9862,10 +9862,10 @@
         <v>118</v>
       </c>
       <c r="Q17" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R17" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
@@ -9918,10 +9918,10 @@
         <v>103</v>
       </c>
       <c r="Q18" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R18" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
@@ -10030,10 +10030,10 @@
         <v>100</v>
       </c>
       <c r="Q20" s="127" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R20" s="127" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
@@ -10089,7 +10089,7 @@
         <v>1</v>
       </c>
       <c r="R21" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.35">
@@ -10198,10 +10198,10 @@
         <v>106</v>
       </c>
       <c r="Q23" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R23" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
@@ -10310,7 +10310,7 @@
         <v>100</v>
       </c>
       <c r="Q25" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R25" s="129" t="s">
         <v>563</v>
@@ -10366,10 +10366,10 @@
         <v>106</v>
       </c>
       <c r="Q26" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R26" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
@@ -10590,10 +10590,10 @@
         <v>68</v>
       </c>
       <c r="Q30" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R30" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
@@ -10646,10 +10646,10 @@
         <v>68</v>
       </c>
       <c r="Q31" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R31" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
@@ -10761,7 +10761,7 @@
         <v>0.93</v>
       </c>
       <c r="R33" s="159" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">
@@ -10814,10 +10814,10 @@
         <v>109</v>
       </c>
       <c r="Q34" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R34" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -10926,10 +10926,10 @@
         <v>103</v>
       </c>
       <c r="Q36" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R36" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.35">
@@ -11038,10 +11038,10 @@
         <v>100</v>
       </c>
       <c r="Q38" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R38" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.35">
@@ -11150,7 +11150,7 @@
         <v>100</v>
       </c>
       <c r="Q40" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R40" s="129" t="s">
         <v>562</v>
@@ -11206,7 +11206,7 @@
         <v>100</v>
       </c>
       <c r="Q41" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R41" s="129" t="s">
         <v>563</v>
@@ -11262,10 +11262,10 @@
         <v>100</v>
       </c>
       <c r="Q42" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R42" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.35">
@@ -11318,10 +11318,10 @@
         <v>100</v>
       </c>
       <c r="Q43" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R43" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.35">
@@ -11374,10 +11374,10 @@
         <v>118</v>
       </c>
       <c r="Q44" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R44" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.35">
@@ -11542,10 +11542,10 @@
         <v>97</v>
       </c>
       <c r="Q47" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R47" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.35">
@@ -11598,10 +11598,10 @@
         <v>97</v>
       </c>
       <c r="Q48" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R48" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.35">
@@ -11710,10 +11710,10 @@
         <v>112</v>
       </c>
       <c r="Q50" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R50" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.35">
@@ -11766,10 +11766,10 @@
         <v>72</v>
       </c>
       <c r="Q51" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R51" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.35">
@@ -11822,10 +11822,10 @@
         <v>72</v>
       </c>
       <c r="Q52" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R52" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.35">
@@ -11878,10 +11878,10 @@
         <v>121</v>
       </c>
       <c r="Q53" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R53" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.35">
@@ -11934,10 +11934,10 @@
         <v>118</v>
       </c>
       <c r="Q54" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R54" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.35">
@@ -12046,10 +12046,10 @@
         <v>103</v>
       </c>
       <c r="Q56" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R56" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.35">
@@ -12158,10 +12158,10 @@
         <v>100</v>
       </c>
       <c r="Q58" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
       <c r="R58" s="129" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.35">
@@ -12273,7 +12273,7 @@
         <v>0.93</v>
       </c>
       <c r="R60" s="159" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.35">
@@ -12329,7 +12329,7 @@
         <v>1</v>
       </c>
       <c r="R61" s="128" t="s">
-        <v>552</v>
+        <v>68</v>
       </c>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.35">

</xml_diff>